<commit_message>
M2: core solver with grid, list and summary output
- CP-SAT model: one Boolean per (home, away, date); a team plays at most once
  per day
- Rules: LEAGUE_BLACKOUT, SEASON_WINDOW, MATCHUP_GAMES, TEAM_GAMES,
  GAMES_PER_DAY, AVAILABILITY, FIXED_GAME, plus Locks; each can be hard or
  soft (weighted penalties in the objective)
- Rule types not implemented yet are reported as not applied
- Output workbook: Grid (home games in the home team's colour, @OPP away),
  List, and Summary with soft violations
- CLI: wildflyer solve
- 2027 example: R18 made soft, since as hard it conflicts with R10 on 7/15
- scripts/bench_scale.py: 30 teams / 150 days solves in ~15s

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KAe16TCDoZ11LwMqHd8H2s
</commit_message>
<xml_diff>
--- a/examples/ausl_2027.xlsx
+++ b/examples/ausl_2027.xlsx
@@ -1361,12 +1361,15 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Hard</t>
-        </is>
+          <t>Soft</t>
+        </is>
+      </c>
+      <c r="P13" t="n">
+        <v>100</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>Only Chicago hosts 7/11-15 (All-Star Weekend travel)</t>
+          <t>Only Chicago hosts 7/11-15 (All-Star Weekend travel). Soft because it conflicts with R10 (Round Rock must host 7/15); as Hard there is no valid schedule</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Series are one opponent at one location
A block (series) was any run of games against one opponent, so 1 away game
plus 2 home games could pass as a 3-game series. A block is now a run of
games against one opponent at one location; a change of host starts a new
block. OPPONENT_BLOCK, REMATCH_GAP, the Checks sheet and the Help text use
the new definition. Regression tests cover mixed-venue series and rematch
gaps between a team's home and away series.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KAe16TCDoZ11LwMqHd8H2s
</commit_message>
<xml_diff>
--- a/examples/ausl_2027.xlsx
+++ b/examples/ausl_2027.xlsx
@@ -5292,7 +5292,7 @@
       </c>
       <c r="B18" s="12" t="inlineStr">
         <is>
-          <t>A run of a team's games against one opponent with no game against anyone else in between. Off days do not break a block.</t>
+          <t>A series: a run of a team's games against one opponent at one location, with no other game in between. Off days do not break a block; a change of location does.</t>
         </is>
       </c>
     </row>
@@ -5617,7 +5617,7 @@
       </c>
       <c r="C31" s="12" t="inlineStr">
         <is>
-          <t>Games against the same opponent come in blocks. A block is a run of a team's games against one opponent with no game against anyone else in between (off days don't break a block). Min/Max = games per block; N = most off days allowed between consecutive games inside a block.</t>
+          <t>Games against the same opponent come in blocks (series). A block is a run of a team's games against one opponent at one location, with no other game in between. Off days don't break a block; a change of location does (home games and away games against the same opponent are separate blocks). Min/Max = games per block; N = most off days allowed between consecutive games inside a block.</t>
         </is>
       </c>
       <c r="D31" s="12" t="inlineStr">

</xml_diff>